<commit_message>
update table 1 formatting
</commit_message>
<xml_diff>
--- a/data/processed/WH01_SuppData_1_deposits_tables.xlsx
+++ b/data/processed/WH01_SuppData_1_deposits_tables.xlsx
@@ -5,37 +5,29 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniofleicester.sharepoint.com/sites/Team_50e7ef44-cf14-4331-9753-a21980019714/Shared Documents/General/Manuscripts &amp; Writing/MS_WongHearing_etal_Ediacaran_Biosphere_Climate/GSABull_submission/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniofleicester.sharepoint.com/sites/Team_50e7ef44-cf14-4331-9753-a21980019714/Shared Documents/General/Manuscripts &amp; Writing/MS_WongHearing_etal_Ediacaran_Biosphere_Climate/Ediacaran_climate_framework/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="8_{886C264E-5784-4BF4-AEEA-DACC98B1B54F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0536CE0-CF3D-426B-B650-2BEE51C165BF}"/>
+  <xr:revisionPtr revIDLastSave="85" documentId="8_{886C264E-5784-4BF4-AEEA-DACC98B1B54F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF0FF68C-F1A0-4EA4-B9A8-5F5D6F35D90F}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-3870" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{5DE8EE72-F8F9-4982-BD2F-826D35F1877B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="3" xr2:uid="{5DE8EE72-F8F9-4982-BD2F-826D35F1877B}"/>
   </bookViews>
   <sheets>
-    <sheet name="references" sheetId="11" state="visible" r:id="rId1"/>
-    <sheet name="csl_deposits" sheetId="13" state="visible" r:id="rId2"/>
-    <sheet name="csl_age_constraints" sheetId="9" state="visible" r:id="rId3"/>
-    <sheet name="Table_1" sheetId="14" state="visible" r:id="rId4"/>
-    <sheet name="Table_4" sheetId="15" state="visible" r:id="rId5"/>
+    <sheet name="references" sheetId="11" r:id="rId1"/>
+    <sheet name="csl_deposits" sheetId="13" r:id="rId2"/>
+    <sheet name="csl_age_constraints" sheetId="9" r:id="rId3"/>
+    <sheet name="Table_1" sheetId="14" r:id="rId4"/>
+    <sheet name="Table_4" sheetId="15" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">csl_age_constraints!$A$1:$AI$212</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">csl_deposits!$A$1:$AP$90</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">references!$A$1:$C$111</definedName>
   </definedNames>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -45,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1508" uniqueCount="1508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9973" uniqueCount="1572">
   <si>
     <t>maximum</t>
   </si>
@@ -4623,15 +4615,207 @@
   <si>
     <t>WH01: ★★★☆☆ rhythmically banded shales (possibly varves), and diamictite with rounded to angular clasts from 3 lithological groups, some of which are facetted.</t>
   </si>
+  <si>
+    <t>compilation</t>
+  </si>
+  <si>
+    <t>Unique deposits</t>
+  </si>
+  <si>
+    <t>Other/Uncertain</t>
+  </si>
+  <si>
+    <t>Retallack (2022)</t>
+  </si>
+  <si>
+    <t>Wang et al. (2023a,b)</t>
+  </si>
+  <si>
+    <t>Niu et al. (2024)</t>
+  </si>
+  <si>
+    <t>Five</t>
+  </si>
+  <si>
+    <t>Four</t>
+  </si>
+  <si>
+    <t>Three</t>
+  </si>
+  <si>
+    <t>Two</t>
+  </si>
+  <si>
+    <t>One</t>
+  </si>
+  <si>
+    <t>Zero</t>
+  </si>
+  <si>
+    <t>Five_pc</t>
+  </si>
+  <si>
+    <t>Four_pc</t>
+  </si>
+  <si>
+    <t>Three_pc</t>
+  </si>
+  <si>
+    <t>Two_pc</t>
+  </si>
+  <si>
+    <t>One_pc</t>
+  </si>
+  <si>
+    <t>Zero_pc</t>
+  </si>
+  <si>
+    <t>Youbi et al. (2020)</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>0 (0 %)</t>
+  </si>
+  <si>
+    <t>10 (40 %)</t>
+  </si>
+  <si>
+    <t>5 (20 %)</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>7 (23 %)</t>
+  </si>
+  <si>
+    <t>3 (10 %)</t>
+  </si>
+  <si>
+    <t>2 (6 %)</t>
+  </si>
+  <si>
+    <t>12 (39 %)</t>
+  </si>
+  <si>
+    <t>Tindal (2023)</t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>84</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>3 (1 %)</t>
+  </si>
+  <si>
+    <t>62 (28 %)</t>
+  </si>
+  <si>
+    <t>84 (38 %)</t>
+  </si>
+  <si>
+    <t>41 (18 %)</t>
+  </si>
+  <si>
+    <t>16 (7 %)</t>
+  </si>
+  <si>
+    <t>18 (8 %)</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>14 (36 %)</t>
+  </si>
+  <si>
+    <t>16 (41 %)</t>
+  </si>
+  <si>
+    <t>5 (13 %)</t>
+  </si>
+  <si>
+    <t>2 (5 %)</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>1 (2 %)</t>
+  </si>
+  <si>
+    <t>16 (32 %)</t>
+  </si>
+  <si>
+    <t>17 (34 %)</t>
+  </si>
+  <si>
+    <t>5 (10 %)</t>
+  </si>
+  <si>
+    <t>3 (6 %)</t>
+  </si>
+  <si>
+    <t>8 (16 %)</t>
+  </si>
+  <si>
+    <t>Gaskiers^1</t>
+  </si>
+  <si>
+    <t>Fauquier^2</t>
+  </si>
+  <si>
+    <t>Bou Azzer^3</t>
+  </si>
+  <si>
+    <t>Hankalchough^4</t>
+  </si>
+  <si>
+    <t>GEG^5</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4737,6 +4921,7 @@
       </fill>
     </dxf>
   </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
       <color rgb="FFFF8282"/>
@@ -5050,7 +5235,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -5059,7 +5244,7 @@
     <col min="3" max="3" width="20.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row customFormat="1" r="1" s="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>527</v>
       </c>
@@ -5070,7 +5255,7 @@
         <v>529</v>
       </c>
     </row>
-    <row customFormat="1" r="2" s="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="12" t="s">
         <v>10</v>
       </c>
@@ -6378,12 +6563,12 @@
     <sortCondition ref="A1:A363"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AP91"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -18091,12 +18276,12 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AI212"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -18134,7 +18319,7 @@
     <col min="35" max="35" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row customFormat="1" r="1" s="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>946</v>
       </c>
@@ -40826,7 +41011,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
@@ -40843,57 +41028,49 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="8.43" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.6328125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>compilation</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Unique deposits</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Gaskiers^a</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Fauquier^b</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Bou Azzer^c</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Hankalchough^d</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>GEG^a</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Other/Uncertain</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Retallack (2022)</t>
-        </is>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>1508</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1509</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1567</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1568</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1569</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1570</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1571</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1511</v>
       </c>
       <c r="B2">
         <v>31</v>
@@ -40917,11 +41094,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Wang et al. (2023a,b)</t>
-        </is>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>1512</v>
       </c>
       <c r="B3">
         <v>39</v>
@@ -40945,11 +41120,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Niu et al. (2024)</t>
-        </is>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>1513</v>
       </c>
       <c r="B4">
         <v>50</v>
@@ -40974,427 +41147,280 @@
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="1" gridLinesSet="1"/>
+  <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M6"/>
-  <sheetFormatPr baseColWidth="8.43" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>compilation</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Five</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Four</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Three</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Two</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>One</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Zero</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Five_pc</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Four_pc</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Three_pc</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Two_pc</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>One_pc</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Zero_pc</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Youbi et al. (2020)</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>0 (0 %)</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>10 (40 %)</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>10 (40 %)</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>5 (20 %)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0 (0 %)</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>0 (0 %)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Retallack (2022)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0 (0 %)</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>7 (23 %)</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>7 (23 %)</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>3 (10 %)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2 (6 %)</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>12 (39 %)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Tindal (2023)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>62</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>3 (1 %)</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>62 (28 %)</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>84 (38 %)</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>41 (18 %)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>16 (7 %)</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>18 (8 %)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Wang et al. (2023a,b)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>0 (0 %)</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>14 (36 %)</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>16 (41 %)</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>5 (13 %)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2 (5 %)</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2 (5 %)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Niu et al. (2024)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>1 (2 %)</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>16 (32 %)</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>17 (34 %)</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>5 (10 %)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>3 (6 %)</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>8 (16 %)</t>
-        </is>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>1508</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1514</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1515</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1516</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1517</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1518</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1519</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1520</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1521</v>
+      </c>
+      <c r="J1" t="s">
+        <v>1522</v>
+      </c>
+      <c r="K1" t="s">
+        <v>1523</v>
+      </c>
+      <c r="L1" t="s">
+        <v>1524</v>
+      </c>
+      <c r="M1" t="s">
+        <v>1525</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1526</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1527</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1528</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1528</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1529</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1527</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1527</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1530</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1531</v>
+      </c>
+      <c r="J2" t="s">
+        <v>1531</v>
+      </c>
+      <c r="K2" t="s">
+        <v>1532</v>
+      </c>
+      <c r="L2" t="s">
+        <v>1530</v>
+      </c>
+      <c r="M2" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>1511</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1527</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1533</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1533</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1534</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1535</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1536</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1530</v>
+      </c>
+      <c r="I3" t="s">
+        <v>1537</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1537</v>
+      </c>
+      <c r="K3" t="s">
+        <v>1538</v>
+      </c>
+      <c r="L3" t="s">
+        <v>1539</v>
+      </c>
+      <c r="M3" t="s">
+        <v>1540</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>1541</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1543</v>
+      </c>
+      <c r="E4" t="s">
+        <v>1544</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1545</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="H4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1548</v>
+      </c>
+      <c r="J4" t="s">
+        <v>1549</v>
+      </c>
+      <c r="K4" t="s">
+        <v>1550</v>
+      </c>
+      <c r="L4" t="s">
+        <v>1551</v>
+      </c>
+      <c r="M4" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>1512</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1527</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1553</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1545</v>
+      </c>
+      <c r="E5" t="s">
+        <v>1529</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1535</v>
+      </c>
+      <c r="G5" t="s">
+        <v>1535</v>
+      </c>
+      <c r="H5" t="s">
+        <v>1530</v>
+      </c>
+      <c r="I5" t="s">
+        <v>1554</v>
+      </c>
+      <c r="J5" t="s">
+        <v>1555</v>
+      </c>
+      <c r="K5" t="s">
+        <v>1556</v>
+      </c>
+      <c r="L5" t="s">
+        <v>1557</v>
+      </c>
+      <c r="M5" t="s">
+        <v>1557</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>1513</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1558</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1545</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1559</v>
+      </c>
+      <c r="E6" t="s">
+        <v>1529</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1534</v>
+      </c>
+      <c r="G6" t="s">
+        <v>1560</v>
+      </c>
+      <c r="H6" t="s">
+        <v>1561</v>
+      </c>
+      <c r="I6" t="s">
+        <v>1562</v>
+      </c>
+      <c r="J6" t="s">
+        <v>1563</v>
+      </c>
+      <c r="K6" t="s">
+        <v>1564</v>
+      </c>
+      <c r="L6" t="s">
+        <v>1565</v>
+      </c>
+      <c r="M6" t="s">
+        <v>1566</v>
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="1" gridLinesSet="1"/>
+  <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100200FB6B67E79FA45AFAC5519C50F741F" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="01717c2105b7b83bf80a64e0903734d8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34f7db31-ae1f-4aec-bd4e-9797ed2b4646" xmlns:ns3="6f64dc32-b692-4574-b8ef-663a628521e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7ce22d48f7aac56f1351f33fc7f5243e" ns2:_="" ns3:_="">
     <xsd:import namespace="34f7db31-ae1f-4aec-bd4e-9797ed2b4646"/>
@@ -41601,15 +41627,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -41622,6 +41639,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B8518A-F80B-496A-A56B-36CEB767A354}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11DF1A6A-5B0D-4AD3-B4C5-C7DE51117ED8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -41636,14 +41661,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B8518A-F80B-496A-A56B-36CEB767A354}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
updates for GSA Bulletin formatting
updating table and figure formatting for GSA Bull proofing
</commit_message>
<xml_diff>
--- a/data/processed/WH01_SuppData_1_deposits_tables.xlsx
+++ b/data/processed/WH01_SuppData_1_deposits_tables.xlsx
@@ -1,43 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniofleicester.sharepoint.com/sites/Team_50e7ef44-cf14-4331-9753-a21980019714/Shared Documents/General/Manuscripts &amp; Writing/MS_WongHearing_etal_Ediacaran_Biosphere_Climate/Ediacaran_climate_framework/data/processed/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniofleicester.sharepoint.com/sites/Team_50e7ef44-cf14-4331-9753-a21980019714/Shared Documents/General/Manuscripts &amp; Writing/MS_accepted_WongHearing_etal_Ediacaran_Biosphere_Climate/Ediacaran_climate_framework/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="85" documentId="8_{886C264E-5784-4BF4-AEEA-DACC98B1B54F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF0FF68C-F1A0-4EA4-B9A8-5F5D6F35D90F}"/>
+  <xr:revisionPtr revIDLastSave="104" documentId="8_{886C264E-5784-4BF4-AEEA-DACC98B1B54F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82508A49-529D-4CAA-A5CC-D9BE4CBE0AEE}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="3" xr2:uid="{5DE8EE72-F8F9-4982-BD2F-826D35F1877B}"/>
+    <workbookView xWindow="-28920" yWindow="-2895" windowWidth="29040" windowHeight="15840" xr2:uid="{5DE8EE72-F8F9-4982-BD2F-826D35F1877B}"/>
   </bookViews>
   <sheets>
-    <sheet name="references" sheetId="11" r:id="rId1"/>
-    <sheet name="csl_deposits" sheetId="13" r:id="rId2"/>
-    <sheet name="csl_age_constraints" sheetId="9" r:id="rId3"/>
-    <sheet name="Table_1" sheetId="14" r:id="rId4"/>
-    <sheet name="Table_4" sheetId="15" r:id="rId5"/>
+    <sheet name="README" sheetId="14" state="visible" r:id="rId1"/>
+    <sheet name="Table_S1_csl_deposits" sheetId="13" state="visible" r:id="rId2"/>
+    <sheet name="Table_S2_csl_age_constraints" sheetId="9" state="visible" r:id="rId3"/>
+    <sheet name="Table_S3_references" sheetId="11" state="visible" r:id="rId4"/>
+    <sheet name="Table_1" sheetId="15" state="visible" r:id="rId5"/>
+    <sheet name="Table_4" sheetId="16" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">csl_age_constraints!$A$1:$AI$212</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">csl_deposits!$A$1:$AP$90</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">references!$A$1:$C$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Table_S1_csl_deposits!$A$1:$AP$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Table_S2_csl_age_constraints!$A$1:$AI$212</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Table_S3_references!$A$1:$C$111</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9973" uniqueCount="1572">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1517" uniqueCount="1517">
   <si>
     <t>maximum</t>
   </si>
@@ -4616,206 +4622,41 @@
     <t>WH01: ★★★☆☆ rhythmically banded shales (possibly varves), and diamictite with rounded to angular clasts from 3 lithological groups, some of which are facetted.</t>
   </si>
   <si>
-    <t>compilation</t>
-  </si>
-  <si>
-    <t>Unique deposits</t>
-  </si>
-  <si>
-    <t>Other/Uncertain</t>
-  </si>
-  <si>
-    <t>Retallack (2022)</t>
-  </si>
-  <si>
-    <t>Wang et al. (2023a,b)</t>
-  </si>
-  <si>
-    <t>Niu et al. (2024)</t>
-  </si>
-  <si>
-    <t>Five</t>
-  </si>
-  <si>
-    <t>Four</t>
-  </si>
-  <si>
-    <t>Three</t>
-  </si>
-  <si>
-    <t>Two</t>
-  </si>
-  <si>
-    <t>One</t>
-  </si>
-  <si>
-    <t>Zero</t>
-  </si>
-  <si>
-    <t>Five_pc</t>
-  </si>
-  <si>
-    <t>Four_pc</t>
-  </si>
-  <si>
-    <t>Three_pc</t>
-  </si>
-  <si>
-    <t>Two_pc</t>
-  </si>
-  <si>
-    <t>One_pc</t>
-  </si>
-  <si>
-    <t>Zero_pc</t>
-  </si>
-  <si>
-    <t>Youbi et al. (2020)</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>0 (0 %)</t>
-  </si>
-  <si>
-    <t>10 (40 %)</t>
-  </si>
-  <si>
-    <t>5 (20 %)</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>7 (23 %)</t>
-  </si>
-  <si>
-    <t>3 (10 %)</t>
-  </si>
-  <si>
-    <t>2 (6 %)</t>
-  </si>
-  <si>
-    <t>12 (39 %)</t>
-  </si>
-  <si>
-    <t>Tindal (2023)</t>
-  </si>
-  <si>
-    <t>62</t>
-  </si>
-  <si>
-    <t>84</t>
-  </si>
-  <si>
-    <t>41</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>3 (1 %)</t>
-  </si>
-  <si>
-    <t>62 (28 %)</t>
-  </si>
-  <si>
-    <t>84 (38 %)</t>
-  </si>
-  <si>
-    <t>41 (18 %)</t>
-  </si>
-  <si>
-    <t>16 (7 %)</t>
-  </si>
-  <si>
-    <t>18 (8 %)</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>14 (36 %)</t>
-  </si>
-  <si>
-    <t>16 (41 %)</t>
-  </si>
-  <si>
-    <t>5 (13 %)</t>
-  </si>
-  <si>
-    <t>2 (5 %)</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>1 (2 %)</t>
-  </si>
-  <si>
-    <t>16 (32 %)</t>
-  </si>
-  <si>
-    <t>17 (34 %)</t>
-  </si>
-  <si>
-    <t>5 (10 %)</t>
-  </si>
-  <si>
-    <t>3 (6 %)</t>
-  </si>
-  <si>
-    <t>8 (16 %)</t>
-  </si>
-  <si>
-    <t>Gaskiers^1</t>
-  </si>
-  <si>
-    <t>Fauquier^2</t>
-  </si>
-  <si>
-    <t>Bou Azzer^3</t>
-  </si>
-  <si>
-    <t>Hankalchough^4</t>
-  </si>
-  <si>
-    <t>GEG^5</t>
+    <t>Worksheet</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Supplementary Data 1: Supplementary geology data file for Wong Hearing et al: Ediacaran coupling of climate and biosphere dynamics</t>
+  </si>
+  <si>
+    <t>Table_S3_references</t>
+  </si>
+  <si>
+    <t>Table_S1_csl_deposits</t>
+  </si>
+  <si>
+    <t>Table_S2_csl_age_constraints</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compilation of the age constraints on each candidate Ediacaran glaciogenic deposit. </t>
+  </si>
+  <si>
+    <t>List of references cited in Supplementary Data 1 tables S1-2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compilation of the candidate Ediacaran glaciogenic deposits considered in this study. For each deposit, the data include deposit synonyms, which compilations a deposit was included in (Youbi et al. 2020; Retallack 2022; Tindal 2023; Wang et al. 2023; Niu et al. 2024), our assessment of their likely glaciogenicity (following Tindal 2023), and our assessment of the most likely interval each deposit is assigned to (MEIH, LEGH, LEIH, TEGH). </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4866,7 +4707,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4897,7 +4738,6 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
@@ -4921,7 +4761,6 @@
       </fill>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
       <color rgb="FFFF8282"/>
@@ -4940,9 +4779,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4980,7 +4819,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -5086,7 +4925,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -5228,1347 +5067,69 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C119"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.08984375" customWidth="1"/>
-    <col min="3" max="3" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.54296875" customWidth="1"/>
+    <col min="2" max="2" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>527</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>528</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>1228</v>
-      </c>
-      <c r="B3">
-        <v>2024</v>
-      </c>
-      <c r="C3" t="s">
-        <v>1320</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>1508</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>1509</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>1103</v>
-      </c>
-      <c r="B4">
-        <v>2011</v>
-      </c>
-      <c r="C4" t="s">
-        <v>1342</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1512</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1516</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>1392</v>
-      </c>
-      <c r="B5">
-        <v>2025</v>
-      </c>
-      <c r="C5" t="s">
-        <v>1391</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1513</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1514</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>1357</v>
-      </c>
-      <c r="B6">
-        <v>1972</v>
-      </c>
-      <c r="C6" t="s">
-        <v>1356</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>338</v>
-      </c>
-      <c r="B7">
-        <v>2019</v>
-      </c>
-      <c r="C7" t="s">
-        <v>1427</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>175</v>
-      </c>
-      <c r="B8">
-        <v>2017</v>
-      </c>
-      <c r="C8" t="s">
-        <v>1428</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>375</v>
-      </c>
-      <c r="B9">
-        <v>2006</v>
-      </c>
-      <c r="C9" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>304</v>
-      </c>
-      <c r="B10">
-        <v>1998</v>
-      </c>
-      <c r="C10" t="s">
-        <v>1429</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>172</v>
-      </c>
-      <c r="B11">
-        <v>1979</v>
-      </c>
-      <c r="C11" t="s">
-        <v>1430</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>315</v>
-      </c>
-      <c r="B12">
-        <v>2005</v>
-      </c>
-      <c r="C12" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>348</v>
-      </c>
-      <c r="B13">
-        <v>2014</v>
-      </c>
-      <c r="C13" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>280</v>
-      </c>
-      <c r="B14">
-        <v>1993</v>
-      </c>
-      <c r="C14" t="s">
-        <v>1307</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>455</v>
-      </c>
-      <c r="B15">
-        <v>2007</v>
-      </c>
-      <c r="C15" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>1262</v>
-      </c>
-      <c r="B16">
-        <v>2023</v>
-      </c>
-      <c r="C16" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>488</v>
-      </c>
-      <c r="B17">
-        <v>2023</v>
-      </c>
-      <c r="C17" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>1354</v>
-      </c>
-      <c r="B18">
-        <v>1981</v>
-      </c>
-      <c r="C18" t="s">
-        <v>1355</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>1348</v>
-      </c>
-      <c r="B19">
-        <v>1984</v>
-      </c>
-      <c r="C19" t="s">
-        <v>1349</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>81</v>
-      </c>
-      <c r="B20">
-        <v>2000</v>
-      </c>
-      <c r="C20" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>80</v>
-      </c>
-      <c r="B21">
-        <v>2004</v>
-      </c>
-      <c r="C21" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>83</v>
-      </c>
-      <c r="B22">
-        <v>2013</v>
-      </c>
-      <c r="C22" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>237</v>
-      </c>
-      <c r="B23">
-        <v>2008</v>
-      </c>
-      <c r="C23" t="s">
-        <v>1431</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24">
-        <v>2009</v>
-      </c>
-      <c r="C24" t="s">
-        <v>1432</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>1299</v>
-      </c>
-      <c r="B25">
-        <v>2011</v>
-      </c>
-      <c r="C25" t="s">
-        <v>1433</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>1300</v>
-      </c>
-      <c r="B26">
-        <v>2011</v>
-      </c>
-      <c r="C26" t="s">
-        <v>1434</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>1297</v>
-      </c>
-      <c r="B27">
-        <v>2011</v>
-      </c>
-      <c r="C27" t="s">
-        <v>1298</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>268</v>
-      </c>
-      <c r="B28">
-        <v>2013</v>
-      </c>
-      <c r="C28" t="s">
-        <v>1435</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>166</v>
-      </c>
-      <c r="B29">
-        <v>2004</v>
-      </c>
-      <c r="C29" t="s">
-        <v>1436</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>128</v>
-      </c>
-      <c r="B30">
-        <v>2011</v>
-      </c>
-      <c r="C30" t="s">
-        <v>1437</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>231</v>
-      </c>
-      <c r="B31">
-        <v>2002</v>
-      </c>
-      <c r="C31" t="s">
-        <v>1361</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>1343</v>
-      </c>
-      <c r="B32">
-        <v>2006</v>
-      </c>
-      <c r="C32" t="s">
-        <v>1344</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>82</v>
-      </c>
-      <c r="B33">
-        <v>2008</v>
-      </c>
-      <c r="C33" t="s">
-        <v>1438</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>354</v>
-      </c>
-      <c r="B34">
-        <v>2021</v>
-      </c>
-      <c r="C34" t="s">
-        <v>1439</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>256</v>
-      </c>
-      <c r="B35">
-        <v>2016</v>
-      </c>
-      <c r="C35" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>376</v>
-      </c>
-      <c r="B36">
-        <v>2010</v>
-      </c>
-      <c r="C36" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>330</v>
-      </c>
-      <c r="B37">
-        <v>2000</v>
-      </c>
-      <c r="C37" t="s">
-        <v>1440</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>39</v>
-      </c>
-      <c r="B38">
-        <v>2023</v>
-      </c>
-      <c r="C38" t="s">
-        <v>1317</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>40</v>
-      </c>
-      <c r="B39">
-        <v>2024</v>
-      </c>
-      <c r="C39" t="s">
-        <v>1318</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>54</v>
-      </c>
-      <c r="B40">
-        <v>2004</v>
-      </c>
-      <c r="C40" t="s">
-        <v>1442</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>48</v>
-      </c>
-      <c r="B41">
-        <v>1998</v>
-      </c>
-      <c r="C41" t="s">
-        <v>1441</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>49</v>
-      </c>
-      <c r="B42">
-        <v>2011</v>
-      </c>
-      <c r="C42" t="s">
-        <v>1443</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>1095</v>
-      </c>
-      <c r="B43">
-        <v>2010</v>
-      </c>
-      <c r="C43" t="s">
-        <v>1312</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>266</v>
-      </c>
-      <c r="B44">
-        <v>2011</v>
-      </c>
-      <c r="C44" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>228</v>
-      </c>
-      <c r="B45">
-        <v>1989</v>
-      </c>
-      <c r="C45" t="s">
-        <v>1360</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>133</v>
-      </c>
-      <c r="B46">
-        <v>2000</v>
-      </c>
-      <c r="C46" t="s">
-        <v>1444</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>405</v>
-      </c>
-      <c r="B47">
-        <v>2015</v>
-      </c>
-      <c r="C47" t="s">
-        <v>1445</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>137</v>
-      </c>
-      <c r="B48">
-        <v>2010</v>
-      </c>
-      <c r="C48" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>436</v>
-      </c>
-      <c r="B49">
-        <v>2006</v>
-      </c>
-      <c r="C49" t="s">
-        <v>1104</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>437</v>
-      </c>
-      <c r="B50">
-        <v>2009</v>
-      </c>
-      <c r="C50" t="s">
-        <v>1105</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>429</v>
-      </c>
-      <c r="B51">
-        <v>2003</v>
-      </c>
-      <c r="C51" t="s">
-        <v>1446</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>424</v>
-      </c>
-      <c r="B52">
-        <v>2004</v>
-      </c>
-      <c r="C52" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>1121</v>
-      </c>
-      <c r="B53">
-        <v>2011</v>
-      </c>
-      <c r="C53" t="s">
-        <v>1447</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
-        <v>167</v>
-      </c>
-      <c r="B54">
-        <v>2008</v>
-      </c>
-      <c r="C54" t="s">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>1194</v>
-      </c>
-      <c r="B55">
-        <v>1981</v>
-      </c>
-      <c r="C55" t="s">
-        <v>1448</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>1129</v>
-      </c>
-      <c r="B56">
-        <v>2017</v>
-      </c>
-      <c r="C56" t="s">
-        <v>1449</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>294</v>
-      </c>
-      <c r="B57">
-        <v>1988</v>
-      </c>
-      <c r="C57" t="s">
-        <v>1450</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>1367</v>
-      </c>
-      <c r="B58">
-        <v>2022</v>
-      </c>
-      <c r="C58" t="s">
-        <v>1366</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
-        <v>73</v>
-      </c>
-      <c r="B59">
-        <v>2024</v>
-      </c>
-      <c r="C59" t="s">
-        <v>1296</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
-        <v>140</v>
-      </c>
-      <c r="B60">
-        <v>2005</v>
-      </c>
-      <c r="C60" t="s">
-        <v>1451</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
-        <v>377</v>
-      </c>
-      <c r="B61">
-        <v>2023</v>
-      </c>
-      <c r="C61" t="s">
-        <v>1452</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
-        <v>245</v>
-      </c>
-      <c r="B62">
-        <v>2018</v>
-      </c>
-      <c r="C62" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
-        <v>60</v>
-      </c>
-      <c r="B63">
-        <v>2018</v>
-      </c>
-      <c r="C63" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
-        <v>158</v>
-      </c>
-      <c r="B64">
-        <v>2022</v>
-      </c>
-      <c r="C64" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
-        <v>287</v>
-      </c>
-      <c r="B65">
-        <v>2007</v>
-      </c>
-      <c r="C65" t="s">
-        <v>1306</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
-        <v>267</v>
-      </c>
-      <c r="B66">
-        <v>2013</v>
-      </c>
-      <c r="C66" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
-        <v>1167</v>
-      </c>
-      <c r="B67">
-        <v>2006</v>
-      </c>
-      <c r="C67" t="s">
-        <v>1453</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
-        <v>382</v>
-      </c>
-      <c r="B68">
-        <v>2015</v>
-      </c>
-      <c r="C68" t="s">
-        <v>1454</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
-        <v>383</v>
-      </c>
-      <c r="B69">
-        <v>2015</v>
-      </c>
-      <c r="C69" t="s">
-        <v>1455</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
-        <v>102</v>
-      </c>
-      <c r="B70">
-        <v>2008</v>
-      </c>
-      <c r="C70" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
-        <v>1166</v>
-      </c>
-      <c r="B71">
-        <v>2015</v>
-      </c>
-      <c r="C71" t="s">
-        <v>1456</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
-        <v>461</v>
-      </c>
-      <c r="B72">
-        <v>2022</v>
-      </c>
-      <c r="C72" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
-        <v>11</v>
-      </c>
-      <c r="B73">
-        <v>2014</v>
-      </c>
-      <c r="C73" t="s">
-        <v>1107</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
-        <v>1478</v>
-      </c>
-      <c r="B74">
-        <v>2007</v>
-      </c>
-      <c r="C74" t="s">
-        <v>1479</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
-        <v>465</v>
-      </c>
-      <c r="B75">
-        <v>2024</v>
-      </c>
-      <c r="C75" t="s">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
-        <v>316</v>
-      </c>
-      <c r="B76">
-        <v>2011</v>
-      </c>
-      <c r="C76" t="s">
-        <v>1310</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
-        <v>116</v>
-      </c>
-      <c r="B77">
-        <v>2019</v>
-      </c>
-      <c r="C77" t="s">
-        <v>1457</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
-        <v>283</v>
-      </c>
-      <c r="B78">
-        <v>2007</v>
-      </c>
-      <c r="C78" t="s">
-        <v>1308</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
-        <v>127</v>
-      </c>
-      <c r="B79">
-        <v>1994</v>
-      </c>
-      <c r="C79" t="s">
-        <v>1426</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
-        <v>1232</v>
-      </c>
-      <c r="B80">
-        <v>2024</v>
-      </c>
-      <c r="C80" t="s">
-        <v>1458</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
-        <v>218</v>
-      </c>
-      <c r="B81">
-        <v>2021</v>
-      </c>
-      <c r="C81" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
-        <v>1346</v>
-      </c>
-      <c r="B82">
-        <v>1964</v>
-      </c>
-      <c r="C82" t="s">
-        <v>1347</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
-        <v>298</v>
-      </c>
-      <c r="B83">
-        <v>2018</v>
-      </c>
-      <c r="C83" t="s">
-        <v>1459</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
-        <v>148</v>
-      </c>
-      <c r="B84">
-        <v>2016</v>
-      </c>
-      <c r="C84" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
-        <v>275</v>
-      </c>
-      <c r="B85">
-        <v>2010</v>
-      </c>
-      <c r="C85" t="s">
-        <v>1460</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
-        <v>362</v>
-      </c>
-      <c r="B86">
-        <v>2015</v>
-      </c>
-      <c r="C86" t="s">
-        <v>1461</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
-        <v>1102</v>
-      </c>
-      <c r="B87">
-        <v>2011</v>
-      </c>
-      <c r="C87" t="s">
-        <v>1311</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
-        <v>29</v>
-      </c>
-      <c r="B88">
-        <v>2014</v>
-      </c>
-      <c r="C88" t="s">
-        <v>1305</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
-        <v>492</v>
-      </c>
-      <c r="B89">
-        <v>2020</v>
-      </c>
-      <c r="C89" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A90" t="s">
-        <v>141</v>
-      </c>
-      <c r="B90">
-        <v>2007</v>
-      </c>
-      <c r="C90" t="s">
-        <v>1462</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
-        <v>142</v>
-      </c>
-      <c r="B91">
-        <v>2011</v>
-      </c>
-      <c r="C91" t="s">
-        <v>1375</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A92" t="s">
-        <v>136</v>
-      </c>
-      <c r="B92">
-        <v>2009</v>
-      </c>
-      <c r="C92" t="s">
-        <v>1463</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
-        <v>38</v>
-      </c>
-      <c r="B93">
-        <v>2023</v>
-      </c>
-      <c r="C93" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A94" t="s">
-        <v>1128</v>
-      </c>
-      <c r="B94">
-        <v>1981</v>
-      </c>
-      <c r="C94" t="s">
-        <v>1464</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A95" t="s">
-        <v>342</v>
-      </c>
-      <c r="B95">
-        <v>2015</v>
-      </c>
-      <c r="C95" t="s">
-        <v>1465</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A96" t="s">
-        <v>411</v>
-      </c>
-      <c r="B96">
-        <v>2002</v>
-      </c>
-      <c r="C96" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
-        <v>391</v>
-      </c>
-      <c r="B97">
-        <v>2000</v>
-      </c>
-      <c r="C97" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
-        <v>176</v>
-      </c>
-      <c r="B98">
-        <v>2023</v>
-      </c>
-      <c r="C98" t="s">
-        <v>1319</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
-        <v>303</v>
-      </c>
-      <c r="B99">
-        <v>1996</v>
-      </c>
-      <c r="C99" t="s">
-        <v>1466</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A100" t="s">
-        <v>100</v>
-      </c>
-      <c r="B100">
-        <v>2013</v>
-      </c>
-      <c r="C100" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A101" t="s">
-        <v>495</v>
-      </c>
-      <c r="B101">
-        <v>2017</v>
-      </c>
-      <c r="C101" t="s">
-        <v>1314</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A102" t="s">
-        <v>109</v>
-      </c>
-      <c r="B102">
-        <v>2020</v>
-      </c>
-      <c r="C102" t="s">
-        <v>1313</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A103" t="s">
-        <v>1184</v>
-      </c>
-      <c r="B103">
-        <v>2021</v>
-      </c>
-      <c r="C103" t="s">
-        <v>1467</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A104" t="s">
-        <v>430</v>
-      </c>
-      <c r="B104">
-        <v>2006</v>
-      </c>
-      <c r="C104" t="s">
-        <v>1106</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A105" t="s">
-        <v>1099</v>
-      </c>
-      <c r="B105">
-        <v>1985</v>
-      </c>
-      <c r="C105" t="s">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A106" t="s">
-        <v>1096</v>
-      </c>
-      <c r="B106">
-        <v>2018</v>
-      </c>
-      <c r="C106" t="s">
-        <v>1469</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A107" t="s">
-        <v>1177</v>
-      </c>
-      <c r="B107">
-        <v>2004</v>
-      </c>
-      <c r="C107" t="s">
-        <v>1470</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A108" t="s">
-        <v>182</v>
-      </c>
-      <c r="B108">
-        <v>2009</v>
-      </c>
-      <c r="C108" t="s">
-        <v>1471</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A109" t="s">
-        <v>31</v>
-      </c>
-      <c r="B109">
-        <v>2021</v>
-      </c>
-      <c r="C109" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A110" t="s">
-        <v>1178</v>
-      </c>
-      <c r="B110">
-        <v>2005</v>
-      </c>
-      <c r="C110" t="s">
-        <v>1472</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A111" t="s">
-        <v>248</v>
-      </c>
-      <c r="B111">
-        <v>2020</v>
-      </c>
-      <c r="C111" t="s">
-        <v>1473</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A112" t="s">
-        <v>1378</v>
-      </c>
-      <c r="B112">
-        <v>2025</v>
-      </c>
-      <c r="C112" t="s">
-        <v>1379</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A113" t="s">
-        <v>121</v>
-      </c>
-      <c r="B113">
-        <v>2017</v>
-      </c>
-      <c r="C113" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A114" t="s">
-        <v>115</v>
-      </c>
-      <c r="B114">
-        <v>2013</v>
-      </c>
-      <c r="C114" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A115" t="s">
-        <v>1483</v>
-      </c>
-      <c r="B115">
-        <v>2025</v>
-      </c>
-      <c r="C115" t="s">
-        <v>1485</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A116" t="s">
-        <v>1484</v>
-      </c>
-      <c r="B116">
-        <v>2025</v>
-      </c>
-      <c r="C116" t="s">
-        <v>1486</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A117" t="s">
-        <v>1487</v>
-      </c>
-      <c r="B117">
-        <v>2024</v>
-      </c>
-      <c r="C117" t="s">
-        <v>1488</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A118" t="s">
-        <v>1491</v>
-      </c>
-      <c r="B118">
-        <v>2026</v>
-      </c>
-      <c r="C118" t="s">
-        <v>1492</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A119" t="s">
-        <v>1501</v>
-      </c>
-      <c r="B119">
-        <v>2021</v>
-      </c>
-      <c r="C119" t="s">
-        <v>1502</v>
+        <v>1511</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1515</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C111" xr:uid="{A1496D4F-A67C-463B-BA28-3CCCE27BB056}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C114">
-      <sortCondition ref="A1:A111"/>
-    </sortState>
-  </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:A363">
-    <sortCondition ref="A1:A363"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:B6">
+    <sortCondition ref="A4:A6"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:AP91"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -18276,12 +16837,12 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:AI212"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -21961,7 +20522,7 @@
       <c r="A35" t="s">
         <v>603</v>
       </c>
-      <c r="B35" s="14" t="s">
+      <c r="B35" s="13" t="s">
         <v>1490</v>
       </c>
       <c r="C35" s="4" t="s">
@@ -40579,7 +39140,7 @@
       <c r="D209" t="s">
         <v>1114</v>
       </c>
-      <c r="E209" s="13" t="s">
+      <c r="E209" s="12" t="s">
         <v>1271</v>
       </c>
       <c r="F209" t="s">
@@ -41011,13 +39572,13 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EF56AFD6-1B00-4726-BE82-44361571D5C3}">
           <x14:formula1>
-            <xm:f>references!$A:$A</xm:f>
+            <xm:f>Table_S3_references!$A:$A</xm:f>
           </x14:formula1>
           <xm:sqref>AF1:AI1048576</xm:sqref>
         </x14:dataValidation>
@@ -41028,49 +39589,1390 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:C119"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.08984375" customWidth="1"/>
+    <col min="3" max="3" width="20.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>1508</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1509</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1567</v>
-      </c>
-      <c r="D1" t="s">
-        <v>1568</v>
-      </c>
-      <c r="E1" t="s">
-        <v>1569</v>
-      </c>
-      <c r="F1" t="s">
-        <v>1570</v>
-      </c>
-      <c r="G1" t="s">
-        <v>1571</v>
-      </c>
-      <c r="H1" t="s">
-        <v>1510</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>1511</v>
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>1228</v>
+      </c>
+      <c r="B3">
+        <v>2024</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1320</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B4">
+        <v>2011</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>1392</v>
+      </c>
+      <c r="B5">
+        <v>2025</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>1357</v>
+      </c>
+      <c r="B6">
+        <v>1972</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1356</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>338</v>
+      </c>
+      <c r="B7">
+        <v>2019</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1427</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>175</v>
+      </c>
+      <c r="B8">
+        <v>2017</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1428</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>375</v>
+      </c>
+      <c r="B9">
+        <v>2006</v>
+      </c>
+      <c r="C9" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>304</v>
+      </c>
+      <c r="B10">
+        <v>1998</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1429</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>172</v>
+      </c>
+      <c r="B11">
+        <v>1979</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>315</v>
+      </c>
+      <c r="B12">
+        <v>2005</v>
+      </c>
+      <c r="C12" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>348</v>
+      </c>
+      <c r="B13">
+        <v>2014</v>
+      </c>
+      <c r="C13" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>280</v>
+      </c>
+      <c r="B14">
+        <v>1993</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1307</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>455</v>
+      </c>
+      <c r="B15">
+        <v>2007</v>
+      </c>
+      <c r="C15" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>1262</v>
+      </c>
+      <c r="B16">
+        <v>2023</v>
+      </c>
+      <c r="C16" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>488</v>
+      </c>
+      <c r="B17">
+        <v>2023</v>
+      </c>
+      <c r="C17" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>1354</v>
+      </c>
+      <c r="B18">
+        <v>1981</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1355</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>1348</v>
+      </c>
+      <c r="B19">
+        <v>1984</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1349</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>81</v>
+      </c>
+      <c r="B20">
+        <v>2000</v>
+      </c>
+      <c r="C20" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21">
+        <v>2004</v>
+      </c>
+      <c r="C21" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>83</v>
+      </c>
+      <c r="B22">
+        <v>2013</v>
+      </c>
+      <c r="C22" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>237</v>
+      </c>
+      <c r="B23">
+        <v>2008</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1431</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>2009</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1432</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>1299</v>
+      </c>
+      <c r="B25">
+        <v>2011</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1433</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>1300</v>
+      </c>
+      <c r="B26">
+        <v>2011</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1434</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>1297</v>
+      </c>
+      <c r="B27">
+        <v>2011</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1298</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>268</v>
+      </c>
+      <c r="B28">
+        <v>2013</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1435</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>166</v>
+      </c>
+      <c r="B29">
+        <v>2004</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1436</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>128</v>
+      </c>
+      <c r="B30">
+        <v>2011</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1437</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>231</v>
+      </c>
+      <c r="B31">
+        <v>2002</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1361</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B32">
+        <v>2006</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>82</v>
+      </c>
+      <c r="B33">
+        <v>2008</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1438</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>354</v>
+      </c>
+      <c r="B34">
+        <v>2021</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>256</v>
+      </c>
+      <c r="B35">
+        <v>2016</v>
+      </c>
+      <c r="C35" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>376</v>
+      </c>
+      <c r="B36">
+        <v>2010</v>
+      </c>
+      <c r="C36" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>330</v>
+      </c>
+      <c r="B37">
+        <v>2000</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38">
+        <v>2023</v>
+      </c>
+      <c r="C38" t="s">
+        <v>1317</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39">
+        <v>2024</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1318</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>54</v>
+      </c>
+      <c r="B40">
+        <v>2004</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>48</v>
+      </c>
+      <c r="B41">
+        <v>1998</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>49</v>
+      </c>
+      <c r="B42">
+        <v>2011</v>
+      </c>
+      <c r="C42" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>1095</v>
+      </c>
+      <c r="B43">
+        <v>2010</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1312</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>266</v>
+      </c>
+      <c r="B44">
+        <v>2011</v>
+      </c>
+      <c r="C44" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>228</v>
+      </c>
+      <c r="B45">
+        <v>1989</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1360</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>133</v>
+      </c>
+      <c r="B46">
+        <v>2000</v>
+      </c>
+      <c r="C46" t="s">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>405</v>
+      </c>
+      <c r="B47">
+        <v>2015</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>137</v>
+      </c>
+      <c r="B48">
+        <v>2010</v>
+      </c>
+      <c r="C48" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>436</v>
+      </c>
+      <c r="B49">
+        <v>2006</v>
+      </c>
+      <c r="C49" t="s">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>437</v>
+      </c>
+      <c r="B50">
+        <v>2009</v>
+      </c>
+      <c r="C50" t="s">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>429</v>
+      </c>
+      <c r="B51">
+        <v>2003</v>
+      </c>
+      <c r="C51" t="s">
+        <v>1446</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>424</v>
+      </c>
+      <c r="B52">
+        <v>2004</v>
+      </c>
+      <c r="C52" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>1121</v>
+      </c>
+      <c r="B53">
+        <v>2011</v>
+      </c>
+      <c r="C53" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>167</v>
+      </c>
+      <c r="B54">
+        <v>2008</v>
+      </c>
+      <c r="C54" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>1194</v>
+      </c>
+      <c r="B55">
+        <v>1981</v>
+      </c>
+      <c r="C55" t="s">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B56">
+        <v>2017</v>
+      </c>
+      <c r="C56" t="s">
+        <v>1449</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>294</v>
+      </c>
+      <c r="B57">
+        <v>1988</v>
+      </c>
+      <c r="C57" t="s">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>1367</v>
+      </c>
+      <c r="B58">
+        <v>2022</v>
+      </c>
+      <c r="C58" t="s">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>73</v>
+      </c>
+      <c r="B59">
+        <v>2024</v>
+      </c>
+      <c r="C59" t="s">
+        <v>1296</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>140</v>
+      </c>
+      <c r="B60">
+        <v>2005</v>
+      </c>
+      <c r="C60" t="s">
+        <v>1451</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>377</v>
+      </c>
+      <c r="B61">
+        <v>2023</v>
+      </c>
+      <c r="C61" t="s">
+        <v>1452</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>245</v>
+      </c>
+      <c r="B62">
+        <v>2018</v>
+      </c>
+      <c r="C62" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>60</v>
+      </c>
+      <c r="B63">
+        <v>2018</v>
+      </c>
+      <c r="C63" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>158</v>
+      </c>
+      <c r="B64">
+        <v>2022</v>
+      </c>
+      <c r="C64" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>287</v>
+      </c>
+      <c r="B65">
+        <v>2007</v>
+      </c>
+      <c r="C65" t="s">
+        <v>1306</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>267</v>
+      </c>
+      <c r="B66">
+        <v>2013</v>
+      </c>
+      <c r="C66" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>1167</v>
+      </c>
+      <c r="B67">
+        <v>2006</v>
+      </c>
+      <c r="C67" t="s">
+        <v>1453</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>382</v>
+      </c>
+      <c r="B68">
+        <v>2015</v>
+      </c>
+      <c r="C68" t="s">
+        <v>1454</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>383</v>
+      </c>
+      <c r="B69">
+        <v>2015</v>
+      </c>
+      <c r="C69" t="s">
+        <v>1455</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>102</v>
+      </c>
+      <c r="B70">
+        <v>2008</v>
+      </c>
+      <c r="C70" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>1166</v>
+      </c>
+      <c r="B71">
+        <v>2015</v>
+      </c>
+      <c r="C71" t="s">
+        <v>1456</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>461</v>
+      </c>
+      <c r="B72">
+        <v>2022</v>
+      </c>
+      <c r="C72" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>11</v>
+      </c>
+      <c r="B73">
+        <v>2014</v>
+      </c>
+      <c r="C73" t="s">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>1478</v>
+      </c>
+      <c r="B74">
+        <v>2007</v>
+      </c>
+      <c r="C74" t="s">
+        <v>1479</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>465</v>
+      </c>
+      <c r="B75">
+        <v>2024</v>
+      </c>
+      <c r="C75" t="s">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>316</v>
+      </c>
+      <c r="B76">
+        <v>2011</v>
+      </c>
+      <c r="C76" t="s">
+        <v>1310</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>116</v>
+      </c>
+      <c r="B77">
+        <v>2019</v>
+      </c>
+      <c r="C77" t="s">
+        <v>1457</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>283</v>
+      </c>
+      <c r="B78">
+        <v>2007</v>
+      </c>
+      <c r="C78" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>127</v>
+      </c>
+      <c r="B79">
+        <v>1994</v>
+      </c>
+      <c r="C79" t="s">
+        <v>1426</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B80">
+        <v>2024</v>
+      </c>
+      <c r="C80" t="s">
+        <v>1458</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>218</v>
+      </c>
+      <c r="B81">
+        <v>2021</v>
+      </c>
+      <c r="C81" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>1346</v>
+      </c>
+      <c r="B82">
+        <v>1964</v>
+      </c>
+      <c r="C82" t="s">
+        <v>1347</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>298</v>
+      </c>
+      <c r="B83">
+        <v>2018</v>
+      </c>
+      <c r="C83" t="s">
+        <v>1459</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>148</v>
+      </c>
+      <c r="B84">
+        <v>2016</v>
+      </c>
+      <c r="C84" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>275</v>
+      </c>
+      <c r="B85">
+        <v>2010</v>
+      </c>
+      <c r="C85" t="s">
+        <v>1460</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>362</v>
+      </c>
+      <c r="B86">
+        <v>2015</v>
+      </c>
+      <c r="C86" t="s">
+        <v>1461</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B87">
+        <v>2011</v>
+      </c>
+      <c r="C87" t="s">
+        <v>1311</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>29</v>
+      </c>
+      <c r="B88">
+        <v>2014</v>
+      </c>
+      <c r="C88" t="s">
+        <v>1305</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>492</v>
+      </c>
+      <c r="B89">
+        <v>2020</v>
+      </c>
+      <c r="C89" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>141</v>
+      </c>
+      <c r="B90">
+        <v>2007</v>
+      </c>
+      <c r="C90" t="s">
+        <v>1462</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>142</v>
+      </c>
+      <c r="B91">
+        <v>2011</v>
+      </c>
+      <c r="C91" t="s">
+        <v>1375</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>136</v>
+      </c>
+      <c r="B92">
+        <v>2009</v>
+      </c>
+      <c r="C92" t="s">
+        <v>1463</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>38</v>
+      </c>
+      <c r="B93">
+        <v>2023</v>
+      </c>
+      <c r="C93" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>1128</v>
+      </c>
+      <c r="B94">
+        <v>1981</v>
+      </c>
+      <c r="C94" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>342</v>
+      </c>
+      <c r="B95">
+        <v>2015</v>
+      </c>
+      <c r="C95" t="s">
+        <v>1465</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>411</v>
+      </c>
+      <c r="B96">
+        <v>2002</v>
+      </c>
+      <c r="C96" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>391</v>
+      </c>
+      <c r="B97">
+        <v>2000</v>
+      </c>
+      <c r="C97" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>176</v>
+      </c>
+      <c r="B98">
+        <v>2023</v>
+      </c>
+      <c r="C98" t="s">
+        <v>1319</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>303</v>
+      </c>
+      <c r="B99">
+        <v>1996</v>
+      </c>
+      <c r="C99" t="s">
+        <v>1466</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>100</v>
+      </c>
+      <c r="B100">
+        <v>2013</v>
+      </c>
+      <c r="C100" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>495</v>
+      </c>
+      <c r="B101">
+        <v>2017</v>
+      </c>
+      <c r="C101" t="s">
+        <v>1314</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>109</v>
+      </c>
+      <c r="B102">
+        <v>2020</v>
+      </c>
+      <c r="C102" t="s">
+        <v>1313</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>1184</v>
+      </c>
+      <c r="B103">
+        <v>2021</v>
+      </c>
+      <c r="C103" t="s">
+        <v>1467</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>430</v>
+      </c>
+      <c r="B104">
+        <v>2006</v>
+      </c>
+      <c r="C104" t="s">
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B105">
+        <v>1985</v>
+      </c>
+      <c r="C105" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>1096</v>
+      </c>
+      <c r="B106">
+        <v>2018</v>
+      </c>
+      <c r="C106" t="s">
+        <v>1469</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>1177</v>
+      </c>
+      <c r="B107">
+        <v>2004</v>
+      </c>
+      <c r="C107" t="s">
+        <v>1470</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>182</v>
+      </c>
+      <c r="B108">
+        <v>2009</v>
+      </c>
+      <c r="C108" t="s">
+        <v>1471</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>31</v>
+      </c>
+      <c r="B109">
+        <v>2021</v>
+      </c>
+      <c r="C109" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>1178</v>
+      </c>
+      <c r="B110">
+        <v>2005</v>
+      </c>
+      <c r="C110" t="s">
+        <v>1472</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
+        <v>248</v>
+      </c>
+      <c r="B111">
+        <v>2020</v>
+      </c>
+      <c r="C111" t="s">
+        <v>1473</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
+        <v>1378</v>
+      </c>
+      <c r="B112">
+        <v>2025</v>
+      </c>
+      <c r="C112" t="s">
+        <v>1379</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>121</v>
+      </c>
+      <c r="B113">
+        <v>2017</v>
+      </c>
+      <c r="C113" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
+        <v>115</v>
+      </c>
+      <c r="B114">
+        <v>2013</v>
+      </c>
+      <c r="C114" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
+        <v>1483</v>
+      </c>
+      <c r="B115">
+        <v>2025</v>
+      </c>
+      <c r="C115" t="s">
+        <v>1485</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>1484</v>
+      </c>
+      <c r="B116">
+        <v>2025</v>
+      </c>
+      <c r="C116" t="s">
+        <v>1486</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
+        <v>1487</v>
+      </c>
+      <c r="B117">
+        <v>2024</v>
+      </c>
+      <c r="C117" t="s">
+        <v>1488</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
+        <v>1491</v>
+      </c>
+      <c r="B118">
+        <v>2026</v>
+      </c>
+      <c r="C118" t="s">
+        <v>1492</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>1501</v>
+      </c>
+      <c r="B119">
+        <v>2021</v>
+      </c>
+      <c r="C119" t="s">
+        <v>1502</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C111" xr:uid="{A1496D4F-A67C-463B-BA28-3CCCE27BB056}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C114">
+      <sortCondition ref="A1:A111"/>
+    </sortState>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:A363">
+    <sortCondition ref="A1:A363"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>compilation</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Unique deposits</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Gaskiers^1</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Fauquier^2</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Bou Azzer^3</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Hankalchough^4</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>GEG^5</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Other/Uncertain</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Retallack (2022)</t>
+        </is>
       </c>
       <c r="B2">
         <v>31</v>
@@ -41094,9 +40996,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>1512</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Wang et al. (2023a,b)</t>
+        </is>
       </c>
       <c r="B3">
         <v>39</v>
@@ -41120,9 +41024,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>1513</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Niu et al. (2024)</t>
+        </is>
       </c>
       <c r="B4">
         <v>50</v>
@@ -41147,280 +41053,427 @@
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="1"/>
+  <printOptions gridLines="1" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>1508</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1514</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1515</v>
-      </c>
-      <c r="D1" t="s">
-        <v>1516</v>
-      </c>
-      <c r="E1" t="s">
-        <v>1517</v>
-      </c>
-      <c r="F1" t="s">
-        <v>1518</v>
-      </c>
-      <c r="G1" t="s">
-        <v>1519</v>
-      </c>
-      <c r="H1" t="s">
-        <v>1520</v>
-      </c>
-      <c r="I1" t="s">
-        <v>1521</v>
-      </c>
-      <c r="J1" t="s">
-        <v>1522</v>
-      </c>
-      <c r="K1" t="s">
-        <v>1523</v>
-      </c>
-      <c r="L1" t="s">
-        <v>1524</v>
-      </c>
-      <c r="M1" t="s">
-        <v>1525</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>1526</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1527</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1528</v>
-      </c>
-      <c r="D2" t="s">
-        <v>1528</v>
-      </c>
-      <c r="E2" t="s">
-        <v>1529</v>
-      </c>
-      <c r="F2" t="s">
-        <v>1527</v>
-      </c>
-      <c r="G2" t="s">
-        <v>1527</v>
-      </c>
-      <c r="H2" t="s">
-        <v>1530</v>
-      </c>
-      <c r="I2" t="s">
-        <v>1531</v>
-      </c>
-      <c r="J2" t="s">
-        <v>1531</v>
-      </c>
-      <c r="K2" t="s">
-        <v>1532</v>
-      </c>
-      <c r="L2" t="s">
-        <v>1530</v>
-      </c>
-      <c r="M2" t="s">
-        <v>1530</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>1511</v>
-      </c>
-      <c r="B3" t="s">
-        <v>1527</v>
-      </c>
-      <c r="C3" t="s">
-        <v>1533</v>
-      </c>
-      <c r="D3" t="s">
-        <v>1533</v>
-      </c>
-      <c r="E3" t="s">
-        <v>1534</v>
-      </c>
-      <c r="F3" t="s">
-        <v>1535</v>
-      </c>
-      <c r="G3" t="s">
-        <v>1536</v>
-      </c>
-      <c r="H3" t="s">
-        <v>1530</v>
-      </c>
-      <c r="I3" t="s">
-        <v>1537</v>
-      </c>
-      <c r="J3" t="s">
-        <v>1537</v>
-      </c>
-      <c r="K3" t="s">
-        <v>1538</v>
-      </c>
-      <c r="L3" t="s">
-        <v>1539</v>
-      </c>
-      <c r="M3" t="s">
-        <v>1540</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>1541</v>
-      </c>
-      <c r="B4" t="s">
-        <v>1534</v>
-      </c>
-      <c r="C4" t="s">
-        <v>1542</v>
-      </c>
-      <c r="D4" t="s">
-        <v>1543</v>
-      </c>
-      <c r="E4" t="s">
-        <v>1544</v>
-      </c>
-      <c r="F4" t="s">
-        <v>1545</v>
-      </c>
-      <c r="G4" t="s">
-        <v>1546</v>
-      </c>
-      <c r="H4" t="s">
-        <v>1547</v>
-      </c>
-      <c r="I4" t="s">
-        <v>1548</v>
-      </c>
-      <c r="J4" t="s">
-        <v>1549</v>
-      </c>
-      <c r="K4" t="s">
-        <v>1550</v>
-      </c>
-      <c r="L4" t="s">
-        <v>1551</v>
-      </c>
-      <c r="M4" t="s">
-        <v>1552</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>1512</v>
-      </c>
-      <c r="B5" t="s">
-        <v>1527</v>
-      </c>
-      <c r="C5" t="s">
-        <v>1553</v>
-      </c>
-      <c r="D5" t="s">
-        <v>1545</v>
-      </c>
-      <c r="E5" t="s">
-        <v>1529</v>
-      </c>
-      <c r="F5" t="s">
-        <v>1535</v>
-      </c>
-      <c r="G5" t="s">
-        <v>1535</v>
-      </c>
-      <c r="H5" t="s">
-        <v>1530</v>
-      </c>
-      <c r="I5" t="s">
-        <v>1554</v>
-      </c>
-      <c r="J5" t="s">
-        <v>1555</v>
-      </c>
-      <c r="K5" t="s">
-        <v>1556</v>
-      </c>
-      <c r="L5" t="s">
-        <v>1557</v>
-      </c>
-      <c r="M5" t="s">
-        <v>1557</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>1513</v>
-      </c>
-      <c r="B6" t="s">
-        <v>1558</v>
-      </c>
-      <c r="C6" t="s">
-        <v>1545</v>
-      </c>
-      <c r="D6" t="s">
-        <v>1559</v>
-      </c>
-      <c r="E6" t="s">
-        <v>1529</v>
-      </c>
-      <c r="F6" t="s">
-        <v>1534</v>
-      </c>
-      <c r="G6" t="s">
-        <v>1560</v>
-      </c>
-      <c r="H6" t="s">
-        <v>1561</v>
-      </c>
-      <c r="I6" t="s">
-        <v>1562</v>
-      </c>
-      <c r="J6" t="s">
-        <v>1563</v>
-      </c>
-      <c r="K6" t="s">
-        <v>1564</v>
-      </c>
-      <c r="L6" t="s">
-        <v>1565</v>
-      </c>
-      <c r="M6" t="s">
-        <v>1566</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>compilation</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Five</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Four</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Three</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Two</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>One</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Zero</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Five_pc</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Four_pc</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Three_pc</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Two_pc</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>One_pc</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Zero_pc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Youbi et al. (2020)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0 (0 %)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>10 (40 %)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>10 (40 %)</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>5 (20 %)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0 (0 %)</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>0 (0 %)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Retallack (2022)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0 (0 %)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>7 (23 %)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>7 (23 %)</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>3 (10 %)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2 (6 %)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>12 (39 %)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Tindal (2023)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>3 (1 %)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>62 (28 %)</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>84 (38 %)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>41 (18 %)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>16 (7 %)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>18 (8 %)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Wang et al. (2023a,b)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0 (0 %)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>14 (36 %)</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>16 (41 %)</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>5 (13 %)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2 (5 %)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2 (5 %)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Niu et al. (2024)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1 (2 %)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>16 (32 %)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>17 (34 %)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>5 (10 %)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>3 (6 %)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>8 (16 %)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="1"/>
+  <printOptions gridLines="1" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100200FB6B67E79FA45AFAC5519C50F741F" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="01717c2105b7b83bf80a64e0903734d8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34f7db31-ae1f-4aec-bd4e-9797ed2b4646" xmlns:ns3="6f64dc32-b692-4574-b8ef-663a628521e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7ce22d48f7aac56f1351f33fc7f5243e" ns2:_="" ns3:_="">
     <xsd:import namespace="34f7db31-ae1f-4aec-bd4e-9797ed2b4646"/>
@@ -41627,6 +41680,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -41639,14 +41701,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B8518A-F80B-496A-A56B-36CEB767A354}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11DF1A6A-5B0D-4AD3-B4C5-C7DE51117ED8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -41661,6 +41715,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B8518A-F80B-496A-A56B-36CEB767A354}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>